<commit_message>
update: apr 2026 settlement full match
</commit_message>
<xml_diff>
--- a/broadway-settlement-apr-2026.xlsx
+++ b/broadway-settlement-apr-2026.xlsx
@@ -2372,10 +2372,10 @@
         <v>474</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>0</v>
+        <v>824046</v>
       </c>
       <c r="L42" s="5" t="n">
-        <v>0</v>
+        <v>807731</v>
       </c>
     </row>
     <row r="43">
@@ -2418,10 +2418,10 @@
         <v>334</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>0</v>
+        <v>580656</v>
       </c>
       <c r="L43" s="5" t="n">
-        <v>0</v>
+        <v>569160</v>
       </c>
     </row>
     <row r="44">
@@ -2464,10 +2464,10 @@
         <v>186</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>0</v>
+        <v>323974</v>
       </c>
       <c r="L44" s="5" t="n">
-        <v>0</v>
+        <v>317560</v>
       </c>
     </row>
     <row r="45">
@@ -2510,10 +2510,10 @@
         <v>266</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>0</v>
+        <v>463318</v>
       </c>
       <c r="L45" s="5" t="n">
-        <v>0</v>
+        <v>454145</v>
       </c>
     </row>
     <row r="47">
@@ -2532,10 +2532,10 @@
         <v>13371.25</v>
       </c>
       <c r="K47" s="8" t="n">
-        <v>21333407</v>
+        <v>23525401</v>
       </c>
       <c r="L47" s="8" t="n">
-        <v>20911021</v>
+        <v>23059617</v>
       </c>
     </row>
     <row r="49">
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1595.47</v>
+        <v>1759.4</v>
       </c>
     </row>
     <row r="50">
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="J50" s="8" t="n">
-        <v>-422386</v>
+        <v>-465784</v>
       </c>
     </row>
     <row r="51">

</xml_diff>

<commit_message>
update: ad cost + final settlement
</commit_message>
<xml_diff>
--- a/broadway-settlement-apr-2026.xlsx
+++ b/broadway-settlement-apr-2026.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="MM/DD/YYYY"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -84,17 +83,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -539,7 +539,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="10" t="n">
         <v>46115</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="10" t="n">
         <v>46116</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="10" t="n">
         <v>46116</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="10" t="n">
         <v>46116</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="10" t="n">
         <v>46116</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="10" t="n">
         <v>46118</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="10" t="n">
         <v>46122</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="10" t="n">
         <v>46123</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="10" t="n">
         <v>46124</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="10" t="n">
         <v>46124</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="10" t="n">
         <v>46125</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="10" t="n">
         <v>46125</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="10" t="n">
         <v>46125</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="10" t="n">
         <v>46126</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="10" t="n">
         <v>46127</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="10" t="n">
         <v>46129</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="10" t="n">
         <v>46130</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="10" t="n">
         <v>46130</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="10" t="n">
         <v>46132</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="10" t="n">
         <v>46132</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="10" t="n">
         <v>46134</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="10" t="n">
         <v>46134</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="10" t="n">
         <v>46134</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" s="10" t="n">
         <v>46135</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" s="10" t="n">
         <v>46135</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
+      <c r="A28" s="10" t="n">
         <v>46135</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
+      <c r="A29" s="10" t="n">
         <v>46136</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" s="10" t="n">
         <v>46136</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="10" t="n">
         <v>46137</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
+      <c r="A32" s="10" t="n">
         <v>46137</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="10" t="n">
         <v>46138</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" s="10" t="n">
         <v>46138</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
+      <c r="A35" s="10" t="n">
         <v>46139</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n">
+      <c r="A36" s="10" t="n">
         <v>46140</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
+      <c r="A37" s="10" t="n">
         <v>46140</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
+      <c r="A38" s="10" t="n">
         <v>46140</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n">
+      <c r="A39" s="10" t="n">
         <v>46142</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
+      <c r="A40" s="10" t="n">
         <v>46142</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
+      <c r="A41" s="10" t="n">
         <v>46142</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n">
+      <c r="A42" s="10" t="n">
         <v>46142</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
+      <c r="A43" s="10" t="n">
         <v>46142</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n">
+      <c r="A44" s="10" t="n">
         <v>46142</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n">
+      <c r="A45" s="10" t="n">
         <v>46142</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -2516,6 +2516,7 @@
         <v>454145</v>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="F47" s="6" t="inlineStr">
         <is>
@@ -2538,6 +2539,7 @@
         <v>23059617</v>
       </c>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
@@ -2579,10 +2581,8 @@
           <t>광고비</t>
         </is>
       </c>
-      <c r="J51" s="9" t="inlineStr">
-        <is>
-          <t>(입력 필요)</t>
-        </is>
+      <c r="J51" s="8" t="n">
+        <v>2264285</v>
       </c>
     </row>
     <row r="52">
@@ -2596,10 +2596,8 @@
           <t>최종 정산금</t>
         </is>
       </c>
-      <c r="J52" s="9" t="inlineStr">
-        <is>
-          <t>(광고비 입력 후 계산)</t>
-        </is>
+      <c r="J52" s="8" t="n">
+        <v>20795332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>